<commit_message>
Revise Huawei application workbooks
</commit_message>
<xml_diff>
--- a/outputs/huawei-permission-application/用户授权路径说明-徒步手表项目填写版.xlsx
+++ b/outputs/huawei-permission-application/用户授权路径说明-徒步手表项目填写版.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rc7f92da374bc4fe3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R42c0bd27528b40d1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -130,13 +130,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="/xl/media/image1.png"/>
+        <xdr:cNvPr id="1" name="/xl/media/image.png"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R4bc128279a984b25"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R37e5e8eeb82e413f"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -326,9 +326,9 @@
 1. 用户打开手机侧徒步 App。
 2. 进入“路线列表”或“导入 GPX”，选择一条徒步路线。
 3. 进入“路线详情”，点击“同步到华为手表”。
-4. App 展示将使用的能力说明：发现已配对华为穿戴设备、读取连接状态/电量/应用安装状态、向手表发送路线数据并接收 ACK/状态消息。
+4. App 展示将使用的华为穿戴能力说明：发现已配对华为穿戴设备、读取连接状态/电量/应用安装状态、向手表发送路线数据并接收 ACK/状态消息。
 5. 用户点击“继续/授权”后，系统或 HMS/Wear Engine 授权弹窗出现；用户同意后才进入设备选择与路线同步。
-6. 如果后续接入 Health Kit / Health Service Kit 读取运动后健康数据，用户需在“设置 -&gt; 健康数据授权”中单独开启，且仅用于本人的运动复盘展示。首轮 Wear Engine 路线同步验证不申请心率、ECG、PPG 等受限人体传感器原始数据。
+6. 如果后续接入 Health Kit / Health Service Kit 读取运动后健康数据，用户需在“设置 -&gt; 健康数据授权”中单独开启，且仅用于本人的运动复盘展示。本次华为申请不申请心率、ECG、PPG 等受限人体传感器原始数据。
 用户修改或撤回授权路径（拟定）：
 1. App 内：设置 -&gt; 设备与数据权限 -&gt; 华为穿戴设备权限，用户可关闭路线同步、设备状态读取或健康数据读取。关闭后，App 不再向华为手表发送新路线，也不再读取对应状态。
 2. 系统内：手机系统设置 -&gt; 应用 -&gt; 本 App -&gt; 权限，关闭蓝牙/附近设备/通知/定位等系统权限。
@@ -350,6 +350,6 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f96578d7d144063"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R63a69cdeaaf243c4"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Fill Huawei application data usage details
</commit_message>
<xml_diff>
--- a/outputs/huawei-permission-application/用户授权路径说明-徒步手表项目填写版.xlsx
+++ b/outputs/huawei-permission-application/用户授权路径说明-徒步手表项目填写版.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R42c0bd27528b40d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R8dedfddabaf24edd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -136,7 +136,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R37e5e8eeb82e413f"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R5d411fc137df4727"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -326,9 +326,12 @@
 1. 用户打开手机侧徒步 App。
 2. 进入“路线列表”或“导入 GPX”，选择一条徒步路线。
 3. 进入“路线详情”，点击“同步到华为手表”。
-4. App 展示将使用的华为穿戴能力说明：发现已配对华为穿戴设备、读取连接状态/电量/应用安装状态、向手表发送路线数据并接收 ACK/状态消息。
+4. App 展示本次同步需要使用的数据和目的：
+   - 设备基础信息：用于识别已配对华为手表、展示设备名称、电量、连接状态、应用安装状态。
+   - 消息通信：用于向手表发送用户选定路线，并接收 ACK、会话状态、偏航状态、低电量状态。
+   - 运动传感器（如申请）：仅用于徒步会话中的运动状态辅助判断和运动后复盘。
 5. 用户点击“继续/授权”后，系统或 HMS/Wear Engine 授权弹窗出现；用户同意后才进入设备选择与路线同步。
-6. 如果后续接入 Health Kit / Health Service Kit 读取运动后健康数据，用户需在“设置 -&gt; 健康数据授权”中单独开启，且仅用于本人的运动复盘展示。本次华为申请不申请心率、ECG、PPG 等受限人体传感器原始数据。
+6. 本次申请不读取睡眠状态、心率、ECG、PPG 等人体传感器原始数据；如后续接入 Health Kit / Health Service Kit 读取健康汇总数据，将在“设置 -&gt; 健康数据授权”中单独说明并请求授权。
 用户修改或撤回授权路径（拟定）：
 1. App 内：设置 -&gt; 设备与数据权限 -&gt; 华为穿戴设备权限，用户可关闭路线同步、设备状态读取或健康数据读取。关闭后，App 不再向华为手表发送新路线，也不再读取对应状态。
 2. 系统内：手机系统设置 -&gt; 应用 -&gt; 本 App -&gt; 权限，关闭蓝牙/附近设备/通知/定位等系统权限。
@@ -350,6 +353,6 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R63a69cdeaaf243c4"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R405411c713674c33"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add heart rate permission to Huawei application
</commit_message>
<xml_diff>
--- a/outputs/huawei-permission-application/用户授权路径说明-徒步手表项目填写版.xlsx
+++ b/outputs/huawei-permission-application/用户授权路径说明-徒步手表项目填写版.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R8dedfddabaf24edd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R15730ad259ed4cf0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -136,7 +136,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R5d411fc137df4727"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R0c87bc9598784924"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -326,18 +326,19 @@
 1. 用户打开手机侧徒步 App。
 2. 进入“路线列表”或“导入 GPX”，选择一条徒步路线。
 3. 进入“路线详情”，点击“同步到华为手表”。
-4. App 展示本次同步需要使用的数据和目的：
+4. App 展示本次同步和徒步记录需要使用的数据和目的：
    - 设备基础信息：用于识别已配对华为手表、展示设备名称、电量、连接状态、应用安装状态。
    - 消息通信：用于向手表发送用户选定路线，并接收 ACK、会话状态、偏航状态、低电量状态。
    - 运动传感器（如申请）：仅用于徒步会话中的运动状态辅助判断和运动后复盘。
-5. 用户点击“继续/授权”后，系统或 HMS/Wear Engine 授权弹窗出现；用户同意后才进入设备选择与路线同步。
-6. 本次申请不读取睡眠状态、心率、ECG、PPG 等人体传感器原始数据；如后续接入 Health Kit / Health Service Kit 读取健康汇总数据，将在“设置 -&gt; 健康数据授权”中单独说明并请求授权。
+   - 心率相关数据：用于徒步中展示当前心率/心率区间，运动后展示心率曲线、平均心率、最高心率和运动负荷参考。
+5. 用户点击“继续/授权”后，系统或 HMS/Wear Engine/Health Kit 授权弹窗出现；用户同意后才进入设备选择、路线同步和徒步心率记录。
+6. 本次不读取睡眠状态、心电图 ECG、PPG 原始波形等非徒步复盘必需数据；心率数据仅用于运动记录和复盘，不用于医疗诊断、疾病筛查或用药建议。
 用户修改或撤回授权路径（拟定）：
-1. App 内：设置 -&gt; 设备与数据权限 -&gt; 华为穿戴设备权限，用户可关闭路线同步、设备状态读取或健康数据读取。关闭后，App 不再向华为手表发送新路线，也不再读取对应状态。
+1. App 内：设置 -&gt; 设备与数据权限 -&gt; 华为穿戴设备权限/健康数据权限，用户可关闭路线同步、设备状态读取、运动传感器或心率数据读取。关闭后，App 不再读取对应数据。
 2. 系统内：手机系统设置 -&gt; 应用 -&gt; 本 App -&gt; 权限，关闭蓝牙/附近设备/通知/定位等系统权限。
-3. HMS / 华为账号相关授权：按华为系统或 HMS Core 授权管理入口撤回相应服务授权。
-4. 撤回后再次使用“同步到华为手表”时，App 会重新说明用途并请求授权。
-截图占位：请补充路线详情页、权限说明页、系统/HMS 授权弹窗、设备选择页、设置撤回授权页截图。</x:v>
+3. HMS / 华为账号 / 健康数据相关授权：按华为系统、HMS Core 或 Health Kit 授权管理入口撤回相应服务授权。
+4. 撤回后再次使用“同步到华为手表”或“记录心率复盘”时，App 会重新说明用途并请求授权。
+截图占位：请补充路线详情页、权限说明页、系统/HMS/Health Kit 授权弹窗、设备选择页、徒步心率展示页、复盘心率曲线页、设置撤回授权页截图。</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -353,6 +354,6 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R405411c713674c33"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc0a0cf464fc4305"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add hiking rest alert scenario to Huawei application
</commit_message>
<xml_diff>
--- a/outputs/huawei-permission-application/用户授权路径说明-徒步手表项目填写版.xlsx
+++ b/outputs/huawei-permission-application/用户授权路径说明-徒步手表项目填写版.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R15730ad259ed4cf0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R73f2823d505c4569"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -136,7 +136,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R0c87bc9598784924"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R5bc8d6b0d7ee43d9"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -328,17 +328,17 @@
 3. 进入“路线详情”，点击“同步到华为手表”。
 4. App 展示本次同步和徒步记录需要使用的数据和目的：
    - 设备基础信息：用于识别已配对华为手表、展示设备名称、电量、连接状态、应用安装状态。
-   - 消息通信：用于向手表发送用户选定路线，并接收 ACK、会话状态、偏航状态、低电量状态。
+   - 消息通信：用于向手表发送用户选定路线，并接收 ACK、会话状态、偏航状态、低电量状态和休息提醒状态。
    - 运动传感器（如申请）：仅用于徒步会话中的运动状态辅助判断和运动后复盘。
-   - 心率相关数据：用于徒步中展示当前心率/心率区间，运动后展示心率曲线、平均心率、最高心率和运动负荷参考。
+   - 心率相关数据：用于徒步中展示当前心率/心率区间；当心率持续处于高强度区间或运动负荷偏高时提醒用户放慢速度、补水或短暂休息；运动后展示心率曲线、平均心率、最高心率、高强度片段和提醒记录。
 5. 用户点击“继续/授权”后，系统或 HMS/Wear Engine/Health Kit 授权弹窗出现；用户同意后才进入设备选择、路线同步和徒步心率记录。
-6. 本次不读取睡眠状态、心电图 ECG、PPG 原始波形等非徒步复盘必需数据；心率数据仅用于运动记录和复盘，不用于医疗诊断、疾病筛查或用药建议。
+6. 本次不读取睡眠状态、心电图 ECG、PPG 原始波形等非徒步场景必需数据；心率数据和休息提醒仅用于运动记录、过程提醒和复盘，不用于医疗诊断、疾病筛查或用药建议。
 用户修改或撤回授权路径（拟定）：
-1. App 内：设置 -&gt; 设备与数据权限 -&gt; 华为穿戴设备权限/健康数据权限，用户可关闭路线同步、设备状态读取、运动传感器或心率数据读取。关闭后，App 不再读取对应数据。
+1. App 内：设置 -&gt; 设备与数据权限 -&gt; 华为穿戴设备权限/健康数据权限，用户可关闭路线同步、设备状态读取、运动传感器、心率数据读取或休息提醒。关闭后，App 不再读取对应数据或生成对应提醒。
 2. 系统内：手机系统设置 -&gt; 应用 -&gt; 本 App -&gt; 权限，关闭蓝牙/附近设备/通知/定位等系统权限。
 3. HMS / 华为账号 / 健康数据相关授权：按华为系统、HMS Core 或 Health Kit 授权管理入口撤回相应服务授权。
-4. 撤回后再次使用“同步到华为手表”或“记录心率复盘”时，App 会重新说明用途并请求授权。
-截图占位：请补充路线详情页、权限说明页、系统/HMS/Health Kit 授权弹窗、设备选择页、徒步心率展示页、复盘心率曲线页、设置撤回授权页截图。</x:v>
+4. 撤回后再次使用“同步到华为手表”“记录心率复盘”或“休息提醒”时，App 会重新说明用途并请求授权。
+截图占位：请补充路线详情页、权限说明页、系统/HMS/Health Kit 授权弹窗、设备选择页、徒步心率展示页、休息提醒页、复盘心率曲线/提醒记录页、设置撤回授权页截图。</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -354,6 +354,6 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc0a0cf464fc4305"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9dea48768b91471c"/>
 </x:worksheet>
 </file>
</xml_diff>